<commit_message>
WIP: review for stratis
</commit_message>
<xml_diff>
--- a/code/vocab_csv/eu-gdpr.xlsx
+++ b/code/vocab_csv/eu-gdpr.xlsx
@@ -3,24 +3,25 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="GDPR_Mapping" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="GDPR_MiscConcepts" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="GDPR_LegalBasis" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="GDPR_LegalBasis_SpecialCategory" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="GDPR_LegalBasis_DataTransfer" sheetId="5" r:id="rId8"/>
-    <sheet state="visible" name="GDPR_LegalRights" sheetId="6" r:id="rId9"/>
-    <sheet state="visible" name="GDPR_LegalRights_Justifications" sheetId="7" r:id="rId10"/>
-    <sheet state="visible" name="GDPR_LegalRights_Impacts" sheetId="8" r:id="rId11"/>
-    <sheet state="visible" name="GDPR_LegalBasis_Rights_Mapping" sheetId="9" r:id="rId12"/>
-    <sheet state="visible" name="GDPR_DataTransfers" sheetId="10" r:id="rId13"/>
-    <sheet state="visible" name="GDPR_DPIA" sheetId="11" r:id="rId14"/>
-    <sheet state="visible" name="GDPR_DPIA_properties" sheetId="12" r:id="rId15"/>
-    <sheet state="visible" name="GDPR_DataBreach" sheetId="13" r:id="rId16"/>
-    <sheet state="visible" name="GDPR_compliance" sheetId="14" r:id="rId17"/>
-    <sheet state="visible" name="GDPR_principles" sheetId="15" r:id="rId18"/>
-    <sheet state="visible" name="GDPR_entities" sheetId="16" r:id="rId19"/>
-    <sheet state="visible" name="GDPR_entities_properties" sheetId="17" r:id="rId20"/>
-    <sheet state="visible" name="GDPR_purpose_compatibility" sheetId="18" r:id="rId21"/>
+    <sheet state="visible" name="GDPR_Mapping" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="GDPR_MiscConcepts" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="GDPR_LegalBasis" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="GDPR_LegalBasis_SpecialCategory" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="GDPR_LegalBasis_DataTransfer" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="GDPR_LegalRights" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="GDPR_LegalRights_Justifications" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="GDPR_LegalRights_Impacts" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="GDPR_LegalBasis_Rights_Mapping" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="GDPR_DataTransfers" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="GDPR_DPIA" sheetId="11" r:id="rId15"/>
+    <sheet state="visible" name="GDPR_DPIA_properties" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="GDPR_DataBreach" sheetId="13" r:id="rId17"/>
+    <sheet state="visible" name="GDPR_compliance" sheetId="14" r:id="rId18"/>
+    <sheet state="visible" name="GDPR_principles" sheetId="15" r:id="rId19"/>
+    <sheet state="visible" name="GDPR_entities" sheetId="16" r:id="rId20"/>
+    <sheet state="visible" name="GDPR_entities_properties" sheetId="17" r:id="rId21"/>
+    <sheet state="visible" name="GDPR_purpose_compatibility" sheetId="18" r:id="rId22"/>
+    <sheet state="visible" name="GDPR_proportionality" sheetId="19" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2591" uniqueCount="1134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2650" uniqueCount="1159">
   <si>
     <t>Concept</t>
   </si>
@@ -372,7 +373,7 @@
     <t>Cross Border Processing</t>
   </si>
   <si>
-    <t>‘Cross-Border Processing’ means either: (a) processing of personal data which takes place in the context of the activities of establishments in more than one Member State of a controller or processor in the Union where the controller or processor is established in more than one Member State; or (b)  processing of personal data which takes place in the context of the activities of a single establishment of a controller or processor in the Union but which substantially affects or is likely to substantially affect data subjects in more than one Member State</t>
+    <t>‘Cross-Border Processing’ means either: (a) processing of personal data which takes place in the context of the activities of establishments in more than one Member State of a controller or processor in the Union where the controller or processor is established in more than one Member State; or (b) processing of personal data which takes place in the context of the activities of a single establishment of a controller or processor in the Union but which substantially affects or is likely to substantially affect data subjects in more than one Member State</t>
   </si>
   <si>
     <t>InformationSocietyService</t>
@@ -3614,13 +3615,13 @@
     <t>Purpose Compatibility</t>
   </si>
   <si>
-    <t>An assessment of the compatbility with a specific Purpose of processing personal data as defined and interpreted under the GDPR</t>
+    <t>Status representing the compatbility with a specific Purpose of processing personal data as defined and interpreted under the GDPR</t>
   </si>
   <si>
     <t>dpv:ReuseCompatibility</t>
   </si>
   <si>
-    <t>Harshvardhan J. Pandit, Georg P. Krog, Julian Flake, Delaram Golpayegani, Beatriz Esteves, Paul Ryan, Arthit Suriyawongkul, Julio Hernandez</t>
+    <t>Harshvardhan J. Pandit, Georg P. Krog, Julian Flake, Delaram Golpayegani, Beatriz Esteves, Paul Ryan, Arthit Suriyawongkul, Julio Hernandez, Stratis Koulierakis</t>
   </si>
   <si>
     <t>PurposeCompatible</t>
@@ -3629,7 +3630,7 @@
     <t>Purpose Compatible</t>
   </si>
   <si>
-    <t>An assessment that the specified use or purpose is compatible with the Purpose of processing personal data as defined and interpreted under the GDPR</t>
+    <t>Status representing the specified use or purpose is compatible with the Purpose of processing personal data as defined and interpreted under the GDPR</t>
   </si>
   <si>
     <t>dpv:PrimaryUse</t>
@@ -3644,10 +3645,85 @@
     <t>Purpose Incompatible</t>
   </si>
   <si>
-    <t>An assessment that the specified use or purpose is incompatible with the Purpose of processing personal data as defined and interpreted under the GDPR</t>
+    <t>Status representing the specified use or purpose is incompatible with the Purpose of processing personal data as defined and interpreted under the GDPR</t>
   </si>
   <si>
     <t>dpv:SecondaryUse</t>
+  </si>
+  <si>
+    <t>PurposeCompatibilityAssessment</t>
+  </si>
+  <si>
+    <t>Purpose Compatibility Assessment</t>
+  </si>
+  <si>
+    <t>An assessment for evaluating the compatibility with the Purpose of processing personal data as defined and interpreted under the GDPR</t>
+  </si>
+  <si>
+    <t>dpv:Assessment</t>
+  </si>
+  <si>
+    <t>ProportionalityAssessment</t>
+  </si>
+  <si>
+    <t>Proportionality Assessment</t>
+  </si>
+  <si>
+    <t>Proportionality is a general principle of EU law, which when applied for the GDPR requires striking a balance between the processing of personal data and the resulting impacts on rights. More simply, the processing should not result in a disproportionate impact on rights</t>
+  </si>
+  <si>
+    <t>dpv:ImpactAssessment</t>
+  </si>
+  <si>
+    <t>The assessment of proportionality requires an assessment of necessity (represented by `eu-gdpr:NecessityAssessment`) and a balancing test (represented by `eu-gdpr:BalancingTest`). The outcome of the proportionality assessment is represented through the `eu-gdpr:ProportionalityStatus` instances</t>
+  </si>
+  <si>
+    <t>Stratis Koulierakis, Georg P. Krog, Harshvardhan J. Pandit</t>
+  </si>
+  <si>
+    <t>NecessityAssessment</t>
+  </si>
+  <si>
+    <t>Necessity Assessment</t>
+  </si>
+  <si>
+    <t>An assessment of whether the processing of personal data is necessary to achieve the stated aims, where necessary indicates a lack of other means which could have been used instead</t>
+  </si>
+  <si>
+    <t>BalancingTest</t>
+  </si>
+  <si>
+    <t>Balancing Test</t>
+  </si>
+  <si>
+    <t>An assessment of whether the individual's interests override the interests of the controller</t>
+  </si>
+  <si>
+    <t>ProportionalityStatus</t>
+  </si>
+  <si>
+    <t>Proportionality Status</t>
+  </si>
+  <si>
+    <t>Status indicating whether the specific activity or context is proportionate</t>
+  </si>
+  <si>
+    <t>dpv:Status</t>
+  </si>
+  <si>
+    <t>Proportionate</t>
+  </si>
+  <si>
+    <t>Status representing the activity or context is proportionate</t>
+  </si>
+  <si>
+    <t>eu-gdpr:ProportionalityStatus</t>
+  </si>
+  <si>
+    <t>Disproportionate</t>
+  </si>
+  <si>
+    <t>Status representing the activity or context is disproportionate i.e. it is not proportionate</t>
   </si>
 </sst>
 </file>
@@ -3891,7 +3967,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="110">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -4176,20 +4252,41 @@
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4288,6 +4385,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -4318,6 +4419,10 @@
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17533,7 +17638,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="17.25"/>
+    <col customWidth="1" min="1" max="2" width="17.25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17593,31 +17698,680 @@
       <c r="AD1" s="97"/>
     </row>
     <row r="2">
-      <c r="A2" s="85" t="s">
+      <c r="A2" s="98" t="s">
         <v>1120</v>
       </c>
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="99" t="s">
         <v>1121</v>
       </c>
+      <c r="C2" s="99" t="s">
+        <v>1122</v>
+      </c>
+      <c r="D2" s="100" t="s">
+        <v>1123</v>
+      </c>
+      <c r="E2" s="100"/>
+      <c r="F2" s="100"/>
+      <c r="G2" s="100"/>
+      <c r="H2" s="100"/>
+      <c r="I2" s="100"/>
+      <c r="J2" s="101">
+        <v>45940.0</v>
+      </c>
+      <c r="K2" s="99" t="s">
+        <v>1124</v>
+      </c>
+      <c r="L2" s="102" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="100"/>
+      <c r="N2" s="100"/>
+      <c r="O2" s="100"/>
+      <c r="P2" s="100"/>
+      <c r="Q2" s="100"/>
+      <c r="R2" s="100"/>
+      <c r="S2" s="100"/>
+      <c r="T2" s="100"/>
+      <c r="U2" s="100"/>
+      <c r="V2" s="100"/>
+      <c r="W2" s="100"/>
+      <c r="X2" s="100"/>
+      <c r="Y2" s="100"/>
+      <c r="Z2" s="100"/>
+      <c r="AA2" s="100"/>
+      <c r="AB2" s="100"/>
+      <c r="AC2" s="100"/>
+      <c r="AD2" s="100"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="103" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B3" s="103" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C3" s="103" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D3" s="100" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E3" s="99" t="s">
+        <v>1129</v>
+      </c>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="101">
+        <v>45940.0</v>
+      </c>
+      <c r="K3" s="99" t="s">
+        <v>1124</v>
+      </c>
+      <c r="L3" s="102" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" s="100"/>
+      <c r="N3" s="100"/>
+      <c r="O3" s="100"/>
+      <c r="P3" s="100"/>
+      <c r="Q3" s="100"/>
+      <c r="R3" s="100"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="100"/>
+      <c r="U3" s="100"/>
+      <c r="V3" s="100"/>
+      <c r="W3" s="100"/>
+      <c r="X3" s="100"/>
+      <c r="Y3" s="100"/>
+      <c r="Z3" s="100"/>
+      <c r="AA3" s="100"/>
+      <c r="AB3" s="100"/>
+      <c r="AC3" s="100"/>
+      <c r="AD3" s="100"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="103" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B4" s="105" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C4" s="103" t="s">
+        <v>1132</v>
+      </c>
+      <c r="D4" s="100" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E4" s="99" t="s">
+        <v>1129</v>
+      </c>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="100"/>
+      <c r="J4" s="101">
+        <v>45940.0</v>
+      </c>
+      <c r="K4" s="99" t="s">
+        <v>1124</v>
+      </c>
+      <c r="L4" s="102" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="100"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="100"/>
+      <c r="P4" s="100"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="100"/>
+      <c r="S4" s="100"/>
+      <c r="T4" s="100"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="100"/>
+      <c r="W4" s="100"/>
+      <c r="X4" s="100"/>
+      <c r="Y4" s="100"/>
+      <c r="Z4" s="100"/>
+      <c r="AA4" s="100"/>
+      <c r="AB4" s="100"/>
+      <c r="AC4" s="100"/>
+      <c r="AD4" s="100"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="102" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B5" s="102" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C5" s="102" t="s">
+        <v>1136</v>
+      </c>
+      <c r="D5" s="102" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E5" s="102" t="s">
+        <v>428</v>
+      </c>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
+      <c r="J5" s="101">
+        <v>45940.0</v>
+      </c>
+      <c r="K5" s="102" t="s">
+        <v>1124</v>
+      </c>
+      <c r="L5" s="102" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="106"/>
+      <c r="N5" s="106"/>
+      <c r="O5" s="106"/>
+      <c r="P5" s="106"/>
+      <c r="Q5" s="106"/>
+      <c r="R5" s="106"/>
+      <c r="S5" s="106"/>
+      <c r="T5" s="106"/>
+      <c r="U5" s="106"/>
+      <c r="V5" s="106"/>
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="106"/>
+      <c r="AB5" s="106"/>
+      <c r="AC5" s="106"/>
+      <c r="AD5" s="106"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="106"/>
+      <c r="B6" s="106"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="106"/>
+      <c r="G6" s="106"/>
+      <c r="H6" s="106"/>
+      <c r="I6" s="106"/>
+      <c r="J6" s="106"/>
+      <c r="K6" s="106"/>
+      <c r="L6" s="106"/>
+      <c r="M6" s="106"/>
+      <c r="N6" s="106"/>
+      <c r="O6" s="106"/>
+      <c r="P6" s="106"/>
+      <c r="Q6" s="106"/>
+      <c r="R6" s="106"/>
+      <c r="S6" s="106"/>
+      <c r="T6" s="106"/>
+      <c r="U6" s="106"/>
+      <c r="V6" s="106"/>
+      <c r="W6" s="106"/>
+      <c r="X6" s="106"/>
+      <c r="Y6" s="106"/>
+      <c r="Z6" s="106"/>
+      <c r="AA6" s="106"/>
+      <c r="AB6" s="106"/>
+      <c r="AC6" s="106"/>
+      <c r="AD6" s="106"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="106"/>
+      <c r="B7" s="106"/>
+      <c r="C7" s="106"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="106"/>
+      <c r="F7" s="106"/>
+      <c r="G7" s="106"/>
+      <c r="H7" s="106"/>
+      <c r="I7" s="106"/>
+      <c r="J7" s="106"/>
+      <c r="K7" s="106"/>
+      <c r="L7" s="106"/>
+      <c r="M7" s="106"/>
+      <c r="N7" s="106"/>
+      <c r="O7" s="106"/>
+      <c r="P7" s="106"/>
+      <c r="Q7" s="106"/>
+      <c r="R7" s="106"/>
+      <c r="S7" s="106"/>
+      <c r="T7" s="106"/>
+      <c r="U7" s="106"/>
+      <c r="V7" s="106"/>
+      <c r="W7" s="106"/>
+      <c r="X7" s="106"/>
+      <c r="Y7" s="106"/>
+      <c r="Z7" s="106"/>
+      <c r="AA7" s="106"/>
+      <c r="AB7" s="106"/>
+      <c r="AC7" s="106"/>
+      <c r="AD7" s="106"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="106"/>
+      <c r="B8" s="106"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="106"/>
+      <c r="M8" s="106"/>
+      <c r="N8" s="106"/>
+      <c r="O8" s="106"/>
+      <c r="P8" s="106"/>
+      <c r="Q8" s="106"/>
+      <c r="R8" s="106"/>
+      <c r="S8" s="106"/>
+      <c r="T8" s="106"/>
+      <c r="U8" s="106"/>
+      <c r="V8" s="106"/>
+      <c r="W8" s="106"/>
+      <c r="X8" s="106"/>
+      <c r="Y8" s="106"/>
+      <c r="Z8" s="106"/>
+      <c r="AA8" s="106"/>
+      <c r="AB8" s="106"/>
+      <c r="AC8" s="106"/>
+      <c r="AD8" s="106"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="106"/>
+      <c r="B9" s="106"/>
+      <c r="C9" s="106"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="106"/>
+      <c r="F9" s="106"/>
+      <c r="G9" s="106"/>
+      <c r="H9" s="106"/>
+      <c r="I9" s="106"/>
+      <c r="J9" s="106"/>
+      <c r="K9" s="106"/>
+      <c r="L9" s="106"/>
+      <c r="M9" s="106"/>
+      <c r="N9" s="106"/>
+      <c r="O9" s="106"/>
+      <c r="P9" s="106"/>
+      <c r="Q9" s="106"/>
+      <c r="R9" s="106"/>
+      <c r="S9" s="106"/>
+      <c r="T9" s="106"/>
+      <c r="U9" s="106"/>
+      <c r="V9" s="106"/>
+      <c r="W9" s="106"/>
+      <c r="X9" s="106"/>
+      <c r="Y9" s="106"/>
+      <c r="Z9" s="106"/>
+      <c r="AA9" s="106"/>
+      <c r="AB9" s="106"/>
+      <c r="AC9" s="106"/>
+      <c r="AD9" s="106"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="106"/>
+      <c r="B10" s="106"/>
+      <c r="C10" s="106"/>
+      <c r="D10" s="106"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
+      <c r="K10" s="106"/>
+      <c r="L10" s="106"/>
+      <c r="M10" s="106"/>
+      <c r="N10" s="106"/>
+      <c r="O10" s="106"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
+      <c r="R10" s="106"/>
+      <c r="S10" s="106"/>
+      <c r="T10" s="106"/>
+      <c r="U10" s="106"/>
+      <c r="V10" s="106"/>
+      <c r="W10" s="106"/>
+      <c r="X10" s="106"/>
+      <c r="Y10" s="106"/>
+      <c r="Z10" s="106"/>
+      <c r="AA10" s="106"/>
+      <c r="AB10" s="106"/>
+      <c r="AC10" s="106"/>
+      <c r="AD10" s="106"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="106"/>
+      <c r="B11" s="106"/>
+      <c r="C11" s="106"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="106"/>
+      <c r="F11" s="106"/>
+      <c r="G11" s="106"/>
+      <c r="H11" s="106"/>
+      <c r="I11" s="106"/>
+      <c r="J11" s="106"/>
+      <c r="K11" s="106"/>
+      <c r="L11" s="106"/>
+      <c r="M11" s="106"/>
+      <c r="N11" s="106"/>
+      <c r="O11" s="106"/>
+      <c r="P11" s="106"/>
+      <c r="Q11" s="106"/>
+      <c r="R11" s="106"/>
+      <c r="S11" s="106"/>
+      <c r="T11" s="106"/>
+      <c r="U11" s="106"/>
+      <c r="V11" s="106"/>
+      <c r="W11" s="106"/>
+      <c r="X11" s="106"/>
+      <c r="Y11" s="106"/>
+      <c r="Z11" s="106"/>
+      <c r="AA11" s="106"/>
+      <c r="AB11" s="106"/>
+      <c r="AC11" s="106"/>
+      <c r="AD11" s="106"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="106"/>
+      <c r="B12" s="106"/>
+      <c r="C12" s="106"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="106"/>
+      <c r="H12" s="106"/>
+      <c r="I12" s="106"/>
+      <c r="J12" s="106"/>
+      <c r="K12" s="106"/>
+      <c r="L12" s="106"/>
+      <c r="M12" s="106"/>
+      <c r="N12" s="106"/>
+      <c r="O12" s="106"/>
+      <c r="P12" s="106"/>
+      <c r="Q12" s="106"/>
+      <c r="R12" s="106"/>
+      <c r="S12" s="106"/>
+      <c r="T12" s="106"/>
+      <c r="U12" s="106"/>
+      <c r="V12" s="106"/>
+      <c r="W12" s="106"/>
+      <c r="X12" s="106"/>
+      <c r="Y12" s="106"/>
+      <c r="Z12" s="106"/>
+      <c r="AA12" s="106"/>
+      <c r="AB12" s="106"/>
+      <c r="AC12" s="106"/>
+      <c r="AD12" s="106"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="106"/>
+      <c r="B13" s="106"/>
+      <c r="C13" s="106"/>
+      <c r="D13" s="106"/>
+      <c r="E13" s="106"/>
+      <c r="F13" s="106"/>
+      <c r="G13" s="106"/>
+      <c r="H13" s="106"/>
+      <c r="I13" s="106"/>
+      <c r="J13" s="106"/>
+      <c r="K13" s="106"/>
+      <c r="L13" s="106"/>
+      <c r="M13" s="106"/>
+      <c r="N13" s="106"/>
+      <c r="O13" s="106"/>
+      <c r="P13" s="106"/>
+      <c r="Q13" s="106"/>
+      <c r="R13" s="106"/>
+      <c r="S13" s="106"/>
+      <c r="T13" s="106"/>
+      <c r="U13" s="106"/>
+      <c r="V13" s="106"/>
+      <c r="W13" s="106"/>
+      <c r="X13" s="106"/>
+      <c r="Y13" s="106"/>
+      <c r="Z13" s="106"/>
+      <c r="AA13" s="106"/>
+      <c r="AB13" s="106"/>
+      <c r="AC13" s="106"/>
+      <c r="AD13" s="106"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="106"/>
+      <c r="B14" s="106"/>
+      <c r="C14" s="106"/>
+      <c r="D14" s="106"/>
+      <c r="E14" s="106"/>
+      <c r="F14" s="106"/>
+      <c r="G14" s="106"/>
+      <c r="H14" s="106"/>
+      <c r="I14" s="106"/>
+      <c r="J14" s="106"/>
+      <c r="K14" s="106"/>
+      <c r="L14" s="106"/>
+      <c r="M14" s="106"/>
+      <c r="N14" s="106"/>
+      <c r="O14" s="106"/>
+      <c r="P14" s="106"/>
+      <c r="Q14" s="106"/>
+      <c r="R14" s="106"/>
+      <c r="S14" s="106"/>
+      <c r="T14" s="106"/>
+      <c r="U14" s="106"/>
+      <c r="V14" s="106"/>
+      <c r="W14" s="106"/>
+      <c r="X14" s="106"/>
+      <c r="Y14" s="106"/>
+      <c r="Z14" s="106"/>
+      <c r="AA14" s="106"/>
+      <c r="AB14" s="106"/>
+      <c r="AC14" s="106"/>
+      <c r="AD14" s="106"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="106"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="106"/>
+      <c r="D15" s="106"/>
+      <c r="E15" s="106"/>
+      <c r="F15" s="106"/>
+      <c r="G15" s="106"/>
+      <c r="H15" s="106"/>
+      <c r="I15" s="106"/>
+      <c r="J15" s="106"/>
+      <c r="K15" s="106"/>
+      <c r="L15" s="106"/>
+      <c r="M15" s="106"/>
+      <c r="N15" s="106"/>
+      <c r="O15" s="106"/>
+      <c r="P15" s="106"/>
+      <c r="Q15" s="106"/>
+      <c r="R15" s="106"/>
+      <c r="S15" s="106"/>
+      <c r="T15" s="106"/>
+      <c r="U15" s="106"/>
+      <c r="V15" s="106"/>
+      <c r="W15" s="106"/>
+      <c r="X15" s="106"/>
+      <c r="Y15" s="106"/>
+      <c r="Z15" s="106"/>
+      <c r="AA15" s="106"/>
+      <c r="AB15" s="106"/>
+      <c r="AC15" s="106"/>
+      <c r="AD15" s="106"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="106"/>
+      <c r="B16" s="106"/>
+      <c r="C16" s="106"/>
+      <c r="D16" s="106"/>
+      <c r="E16" s="106"/>
+      <c r="F16" s="106"/>
+      <c r="G16" s="106"/>
+      <c r="H16" s="106"/>
+      <c r="I16" s="106"/>
+      <c r="J16" s="106"/>
+      <c r="K16" s="106"/>
+      <c r="L16" s="106"/>
+      <c r="M16" s="106"/>
+      <c r="N16" s="106"/>
+      <c r="O16" s="106"/>
+      <c r="P16" s="106"/>
+      <c r="Q16" s="106"/>
+      <c r="R16" s="106"/>
+      <c r="S16" s="106"/>
+      <c r="T16" s="106"/>
+      <c r="U16" s="106"/>
+      <c r="V16" s="106"/>
+      <c r="W16" s="106"/>
+      <c r="X16" s="106"/>
+      <c r="Y16" s="106"/>
+      <c r="Z16" s="106"/>
+      <c r="AA16" s="106"/>
+      <c r="AB16" s="106"/>
+      <c r="AC16" s="106"/>
+      <c r="AD16" s="106"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="106"/>
+      <c r="B17" s="106"/>
+      <c r="C17" s="106"/>
+      <c r="D17" s="106"/>
+      <c r="E17" s="106"/>
+      <c r="F17" s="106"/>
+      <c r="G17" s="106"/>
+      <c r="H17" s="106"/>
+      <c r="I17" s="106"/>
+      <c r="J17" s="106"/>
+      <c r="K17" s="106"/>
+      <c r="L17" s="106"/>
+      <c r="M17" s="106"/>
+      <c r="N17" s="106"/>
+      <c r="O17" s="106"/>
+      <c r="P17" s="106"/>
+      <c r="Q17" s="106"/>
+      <c r="R17" s="106"/>
+      <c r="S17" s="106"/>
+      <c r="T17" s="106"/>
+      <c r="U17" s="106"/>
+      <c r="V17" s="106"/>
+      <c r="W17" s="106"/>
+      <c r="X17" s="106"/>
+      <c r="Y17" s="106"/>
+      <c r="Z17" s="106"/>
+      <c r="AA17" s="106"/>
+      <c r="AB17" s="106"/>
+      <c r="AC17" s="106"/>
+      <c r="AD17" s="106"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="17.25"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="93" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="93" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="94" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="95" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="95" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" s="95" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="95" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" s="95" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="95" t="s">
+        <v>80</v>
+      </c>
+      <c r="J1" s="96" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="95" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="95" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>1139</v>
+      </c>
       <c r="C2" s="50" t="s">
-        <v>1122</v>
-      </c>
-      <c r="D2" s="51" t="s">
-        <v>1123</v>
-      </c>
-      <c r="E2" s="51"/>
+        <v>1140</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>428</v>
+      </c>
       <c r="F2" s="51"/>
       <c r="G2" s="51"/>
       <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="98">
-        <v>45827.0</v>
-      </c>
-      <c r="K2" s="51" t="s">
-        <v>1124</v>
-      </c>
-      <c r="L2" s="51" t="s">
-        <v>204</v>
+      <c r="I2" s="50" t="s">
+        <v>1142</v>
+      </c>
+      <c r="J2" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K2" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L2" s="50" t="s">
+        <v>11</v>
       </c>
       <c r="M2" s="51"/>
       <c r="N2" s="51"/>
@@ -17639,33 +18393,33 @@
       <c r="AD2" s="51"/>
     </row>
     <row r="3">
-      <c r="A3" s="99" t="s">
-        <v>1125</v>
-      </c>
-      <c r="B3" s="99" t="s">
-        <v>1126</v>
-      </c>
-      <c r="C3" s="100" t="s">
-        <v>1127</v>
-      </c>
-      <c r="D3" s="51" t="s">
-        <v>1128</v>
+      <c r="A3" s="8" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C3" s="103" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>1137</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>1129</v>
+        <v>428</v>
       </c>
       <c r="F3" s="51"/>
       <c r="G3" s="51"/>
-      <c r="H3" s="101"/>
+      <c r="H3" s="108"/>
       <c r="I3" s="51"/>
-      <c r="J3" s="98">
-        <v>45827.0</v>
-      </c>
-      <c r="K3" s="51" t="s">
-        <v>1124</v>
-      </c>
-      <c r="L3" s="90" t="s">
-        <v>204</v>
+      <c r="J3" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K3" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L3" s="50" t="s">
+        <v>11</v>
       </c>
       <c r="M3" s="51"/>
       <c r="N3" s="51"/>
@@ -17687,33 +18441,33 @@
       <c r="AD3" s="51"/>
     </row>
     <row r="4">
-      <c r="A4" s="99" t="s">
-        <v>1130</v>
-      </c>
-      <c r="B4" s="102" t="s">
-        <v>1131</v>
-      </c>
-      <c r="C4" s="100" t="s">
-        <v>1132</v>
-      </c>
-      <c r="D4" s="51" t="s">
-        <v>1133</v>
+      <c r="A4" s="8" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C4" s="109" t="s">
+        <v>1149</v>
+      </c>
+      <c r="D4" s="50" t="s">
+        <v>1137</v>
       </c>
       <c r="E4" s="50" t="s">
-        <v>1129</v>
+        <v>428</v>
       </c>
       <c r="F4" s="51"/>
       <c r="G4" s="51"/>
-      <c r="H4" s="101"/>
+      <c r="H4" s="108"/>
       <c r="I4" s="51"/>
-      <c r="J4" s="98">
-        <v>45827.0</v>
-      </c>
-      <c r="K4" s="51" t="s">
-        <v>1124</v>
-      </c>
-      <c r="L4" s="90" t="s">
-        <v>204</v>
+      <c r="J4" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K4" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L4" s="50" t="s">
+        <v>11</v>
       </c>
       <c r="M4" s="51"/>
       <c r="N4" s="51"/>
@@ -17733,6 +18487,98 @@
       <c r="AB4" s="51"/>
       <c r="AC4" s="51"/>
       <c r="AD4" s="51"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C5" s="109" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D5" s="51"/>
+      <c r="E5" s="50" t="s">
+        <v>1153</v>
+      </c>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K5" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L5" s="50" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="51"/>
+      <c r="N5" s="51"/>
+      <c r="O5" s="51"/>
+      <c r="P5" s="51"/>
+      <c r="Q5" s="51"/>
+      <c r="R5" s="51"/>
+      <c r="S5" s="51"/>
+      <c r="T5" s="51"/>
+      <c r="U5" s="51"/>
+      <c r="V5" s="51"/>
+      <c r="W5" s="51"/>
+      <c r="X5" s="51"/>
+      <c r="Y5" s="51"/>
+      <c r="Z5" s="51"/>
+      <c r="AA5" s="51"/>
+      <c r="AB5" s="51"/>
+      <c r="AC5" s="51"/>
+      <c r="AD5" s="51"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>1156</v>
+      </c>
+      <c r="J6" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K6" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L6" s="50" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>1156</v>
+      </c>
+      <c r="J7" s="107">
+        <v>45940.0</v>
+      </c>
+      <c r="K7" s="50" t="s">
+        <v>1143</v>
+      </c>
+      <c r="L7" s="50" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>